<commit_message>
v0.1: feat(edim-web): dense(B) 기반 CPQ·PLM 프론트엔드 1차 — 셸(MDI·F-key)·5화면·mock API
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_컴포넌트정의서.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_컴포넌트정의서.xlsx
@@ -71,12 +71,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3C4"/>
+        <fgColor rgb="00E8F4FD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F4FD"/>
+        <fgColor rgb="00FFF3C4"/>
       </patternFill>
     </fill>
     <fill>
@@ -159,10 +159,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -811,14 +811,14 @@
           <t>P1~</t>
         </is>
       </c>
-      <c r="K2" s="8" t="inlineStr">
-        <is>
-          <t>프로토타입 배포</t>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>구축중</t>
         </is>
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>https://edim.seekerslab.com — Drawing Viewer·DXF/IFC 업로드·AI 생성(샘플 모드)</t>
+          <t>edim-web(React19+Vite+TS, dense B안) — /cpq 셸(MDI·F-key·메뉴트리)·제품선정·기술데이터·Run, mock API(OpenAPI 대응). 루트(/)는 Drawing Viewer 프로토타입 유지</t>
         </is>
       </c>
     </row>
@@ -873,10 +873,14 @@
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>미착수</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="inlineStr"/>
+          <t>구축중</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>edim-web /plm — Design Editor(CAD 툴바·파라메트릭 치수·커맨드라인)·Work Process(MAKE/BUY) — mock API</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -1055,7 +1059,7 @@
           <t>GW-01</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>게이트웨이</t>
         </is>
@@ -1095,7 +1099,7 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="K7" s="8" t="inlineStr">
+      <c r="K7" s="9" t="inlineStr">
         <is>
           <t>개발 대체 구축</t>
         </is>
@@ -1115,7 +1119,7 @@
           <t>SVC-01</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>게이트웨이</t>
         </is>
@@ -2915,7 +2919,7 @@
           <t>P1</t>
         </is>
       </c>
-      <c r="K39" s="8" t="inlineStr">
+      <c r="K39" s="9" t="inlineStr">
         <is>
           <t>부분 구축</t>
         </is>

</xml_diff>

<commit_message>
v0.2: feat(edim-web): Code Set-up·ERP 8화면 추가 (13화면·4모듈) — 게이트웨이 인증 일원화(앱 로그인 제거), basic auth edim
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_컴포넌트정의서.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_컴포넌트정의서.xlsx
@@ -818,7 +818,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>edim-web(React19+Vite+TS, dense B안) — /cpq 셸(MDI·F-key·메뉴트리)·제품선정·기술데이터·Run, mock API(OpenAPI 대응). 루트(/)는 Drawing Viewer 프로토타입 유지</t>
+          <t>edim-web(React19+Vite+TS, dense B안) — 셸(4모듈·MDI·F-key)·CPQ 3화면·ERP 5화면(Project·Dashboard·단가·Process·구매발주), mock API(OpenAPI 대응). 루트(/)는 Drawing Viewer 프로토타입 유지</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
-          <t>edim-web /plm — Design Editor(CAD 툴바·파라메트릭 치수·커맨드라인)·Work Process(MAKE/BUY) — mock API</t>
+          <t>edim-web — Design Editor·Work Process(/plm) + Code Set-up 3화면(/code: Sub Code·Relationship Running Test·데이터 Table) — mock API</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v0.5: feat(edim-web): all 24 wireframe screens — Toolbox(MacroStudio 4-way, UI Designer) + common(approval/tasks/folder/mobile) + docmgmt/doctpl/print/duct/access; MDI scrollbar fix
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_컴포넌트정의서.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_컴포넌트정의서.xlsx
@@ -818,7 +818,7 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>edim-web(React19+Vite+TS, dense B안) — 셸(4모듈·MDI·F-key)·CPQ 3화면·ERP 5화면(Project·Dashboard·단가·Process·구매발주), mock API(OpenAPI 대응). 루트(/)는 Drawing Viewer 프로토타입 유지</t>
+          <t>edim-web(React19+Vite+TS, dense B안) — 6모듈 셸(MDI·F-key), 와이어프레임 24화면 전량 + 상세 드릴다운 4종, mock API(OpenAPI 대응). 루트(/)는 Drawing Viewer 프로토타입 유지</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
-          <t>edim-web — Design Editor·Work Process(/plm) + Code Set-up 3화면(/code: Sub Code·Relationship Running Test·데이터 Table) — mock API</t>
+          <t>edim-web /code·/plm — Sub Code·Relationship(Running Test)·데이터 Table·Design Editor·Work Process·Duct — mock API</t>
         </is>
       </c>
     </row>
@@ -933,10 +933,14 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>미착수</t>
-        </is>
-      </c>
-      <c r="L4" s="7" t="inlineStr"/>
+          <t>구축중</t>
+        </is>
+      </c>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>edim-web /toolbox — Macro Studio(4-Way Sync·TESTED 게이트)·UI Designer(팔레트·Inspector·AI 초안) — mock</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">

</xml_diff>

<commit_message>
v0.6: docs: real-backend integration status (SVC-01/03/05/07/08 구축중, live E2E)
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_컴포넌트정의서.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_컴포넌트정의서.xlsx
@@ -1165,10 +1165,14 @@
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>미착수</t>
-        </is>
-      </c>
-      <c r="L8" s="7" t="inlineStr"/>
+          <t>구축중</t>
+        </is>
+      </c>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>/api/v1/auth/login — sys_user 실검증(sha256)·HMAC 토큰</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
@@ -1277,10 +1281,14 @@
       </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>미착수</t>
-        </is>
-      </c>
-      <c r="L10" s="7" t="inlineStr"/>
+          <t>구축중</t>
+        </is>
+      </c>
+      <c r="L10" s="7" t="inlineStr">
+        <is>
+          <t>/api/v1 codes — group slots·BOM expand(재귀 CTE+slot_map, 실 PG)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
@@ -1393,10 +1401,14 @@
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>미착수</t>
-        </is>
-      </c>
-      <c r="L12" s="7" t="inlineStr"/>
+          <t>구축중</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>/api/v1/tables/tech-data — tbl_data_row(row_key_num) 조회</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
@@ -1505,10 +1517,14 @@
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>미착수</t>
-        </is>
-      </c>
-      <c r="L14" s="7" t="inlineStr"/>
+          <t>구축중</t>
+        </is>
+      </c>
+      <c r="L14" s="7" t="inlineStr">
+        <is>
+          <t>/api/v1/cpq/runs — 202+폴링, cpq_run/cpq_output 영속 (파이프라인 단계는 mock)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -1561,10 +1577,14 @@
       </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>미착수</t>
-        </is>
-      </c>
-      <c r="L15" s="7" t="inlineStr"/>
+          <t>구축중</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>/api/v1/prices/resolve — cst_price 우선순위 resolve(APPLIED→…→QUOTE)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">

</xml_diff>